<commit_message>
update daily dashboard 2026-07-25
</commit_message>
<xml_diff>
--- a/每日输出/小短/郑州-小短-每日风灵不在线.xlsx
+++ b/每日输出/小短/郑州-小短-每日风灵不在线.xlsx
@@ -605,7 +605,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1688856396700701</t>
+          <t>1688854644796118</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -615,22 +615,22 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>李丹阳战队</t>
+          <t>王梦迪战队</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>张亚丽</t>
+          <t>张昱莹</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>zhangyali</t>
+          <t>zhangyuying01</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -642,7 +642,12 @@
         <v>1</v>
       </c>
       <c r="O2" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
+        </is>
       </c>
       <c r="Q2" t="n">
         <v>1</v>
@@ -684,7 +689,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1688858172724149</t>
+          <t>1688856448789579</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -694,22 +699,22 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>吕志恒战队</t>
+          <t>仵夏炎战队</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>吕志恒</t>
+          <t>仵夏炎</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>lvzhiheng</t>
+          <t>wuxiayan</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -763,7 +768,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1688855425700511</t>
+          <t>1688858040865393</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -773,22 +778,22 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>李丹阳战队</t>
+          <t>仵夏炎战队</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>李丹阳</t>
+          <t>王欣冉</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>lidanyang</t>
+          <t>wangxinran</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -842,7 +847,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1688855861872405</t>
+          <t>1688854426767496</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -852,22 +857,22 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>魏新卓战队</t>
+          <t>李少辉战队</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>张碧玉</t>
+          <t>杨喜菊</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>zhangbiyu</t>
+          <t>yangxiju</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -879,12 +884,7 @@
         <v>1</v>
       </c>
       <c r="O5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
-        </is>
+        <v>1</v>
       </c>
       <c r="Q5" t="n">
         <v>1</v>
@@ -926,7 +926,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1688854876688129</t>
+          <t>1688858172724149</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -936,22 +936,22 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>王梦迪战队</t>
+          <t>吕志恒战队</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>王梦迪</t>
+          <t>吕志恒</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>wangmengdi01</t>
+          <t>lvzhiheng</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -1005,7 +1005,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>1688856390786280</t>
+          <t>1688854644796116</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1020,17 +1020,17 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>周莹莹</t>
+          <t>荆雅博</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>zhouyingying01</t>
+          <t>jingyabo</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -1084,7 +1084,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>1688854426767496</t>
+          <t>1688857053845933</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1094,22 +1094,22 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>李少辉战队</t>
+          <t>仵夏炎战队</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>杨喜菊</t>
+          <t>裴芳</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>yangxiju</t>
+          <t>peifang</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>1688856448789579</t>
+          <t>1688855001729445</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1173,22 +1173,22 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>仵夏炎战队</t>
+          <t>李少辉战队</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>仵夏炎</t>
+          <t>李少辉</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>wuxiayan</t>
+          <t>lishaohui</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1197,13 +1197,28 @@
         </is>
       </c>
       <c r="M9" t="n">
-        <v>1</v>
+        <v>0.9444444444444444</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
       </c>
       <c r="O9" t="n">
-        <v>1</v>
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>6,7,8,9,10,11</t>
+        </is>
       </c>
       <c r="Q9" t="n">
-        <v>1</v>
+        <v>0.9444444444444444</v>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
@@ -1242,7 +1257,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>1688857053845933</t>
+          <t>1688857317798186</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1257,17 +1272,17 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>裴芳</t>
+          <t>樊思路</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>peifang</t>
+          <t>fansilu</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1321,7 +1336,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>1688854644796118</t>
+          <t>1688856390786280</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1331,22 +1346,22 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>王梦迪战队</t>
+          <t>仵夏炎战队</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>张昱莹</t>
+          <t>周莹莹</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>zhangyuying01</t>
+          <t>zhouyingying01</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1358,12 +1373,7 @@
         <v>1</v>
       </c>
       <c r="O11" t="n">
-        <v>0</v>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
-        </is>
+        <v>1</v>
       </c>
       <c r="Q11" t="n">
         <v>1</v>
@@ -1405,7 +1415,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1688854644796116</t>
+          <t>1688856396700701</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1415,22 +1425,22 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>仵夏炎战队</t>
+          <t>李丹阳战队</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>荆雅博</t>
+          <t>张亚丽</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>jingyabo</t>
+          <t>zhangyali</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1484,7 +1494,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1688854397763628</t>
+          <t>1688854876688129</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1494,22 +1504,22 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>李少辉战队</t>
+          <t>王梦迪战队</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>李京哲</t>
+          <t>王梦迪</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>lijingzhe</t>
+          <t>wangmengdi01</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1563,7 +1573,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1688858040865393</t>
+          <t>1688855425700511</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1573,22 +1583,22 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>仵夏炎战队</t>
+          <t>李丹阳战队</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>王欣冉</t>
+          <t>李丹阳</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>wangxinran</t>
+          <t>lidanyang</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1642,7 +1652,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1688854619909919</t>
+          <t>1688856227810743</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1652,22 +1662,22 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>吕志恒战队</t>
+          <t>仵夏炎战队</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>刘栋辉</t>
+          <t>陈湘茹</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>liudonghui</t>
+          <t>chenxiangru</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1679,15 +1689,15 @@
         <v>1</v>
       </c>
       <c r="O15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
-        </is>
+        <v>1</v>
       </c>
       <c r="Q15" t="n">
-        <v>1</v>
+        <v>0.7777777777777778</v>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>6,7,8,9</t>
+        </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
@@ -1726,7 +1736,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>1688856227810743</t>
+          <t>1688855861872405</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1736,22 +1746,22 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>仵夏炎战队</t>
+          <t>吕志恒战队</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>陈湘茹</t>
+          <t>张碧玉</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>chenxiangru</t>
+          <t>zhangbiyu</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1763,7 +1773,12 @@
         <v>1</v>
       </c>
       <c r="O16" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
+        </is>
       </c>
       <c r="Q16" t="n">
         <v>1</v>
@@ -1805,7 +1820,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>1688855001729445</t>
+          <t>1688857047874555</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1815,22 +1830,22 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>李少辉战队</t>
+          <t>仵夏炎战队</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>李少辉</t>
+          <t>王常菲</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>lishaohui</t>
+          <t>wangchangfei</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1842,7 +1857,12 @@
         <v>1</v>
       </c>
       <c r="O17" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
+        </is>
       </c>
       <c r="Q17" t="n">
         <v>1</v>
@@ -1884,7 +1904,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>1688857317798186</t>
+          <t>未上报</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1899,17 +1919,17 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>樊思路</t>
+          <t>秦淑楠</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>fansilu</t>
+          <t>qinshunan</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1918,13 +1938,28 @@
         </is>
       </c>
       <c r="M18" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
+        </is>
       </c>
       <c r="O18" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
+        </is>
       </c>
       <c r="Q18" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
+        </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
@@ -1963,7 +1998,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>未上报</t>
+          <t>1688854397763628</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1973,22 +2008,22 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>仵夏炎战队</t>
+          <t>李少辉战队</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>秦淑楠</t>
+          <t>李京哲</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>qinshunan</t>
+          <t>lijingzhe</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -1997,28 +2032,13 @@
         </is>
       </c>
       <c r="M19" t="n">
-        <v>0</v>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
-        </is>
+        <v>1</v>
       </c>
       <c r="O19" t="n">
-        <v>0</v>
-      </c>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
-        </is>
+        <v>1</v>
       </c>
       <c r="Q19" t="n">
-        <v>0</v>
-      </c>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
-        </is>
+        <v>1</v>
       </c>
       <c r="S19" t="inlineStr">
         <is>
@@ -2057,7 +2077,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>1688857047874555</t>
+          <t>1688854619909919</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2067,22 +2087,22 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>仵夏炎战队</t>
+          <t>吕志恒战队</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>王常菲</t>
+          <t>刘栋辉</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>wangchangfei</t>
+          <t>liudonghui</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -2207,7 +2227,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2232,17 +2252,17 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>王梦迪战队</t>
+          <t>李丹阳战队</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>zhangyuying01</t>
+          <t>lidanyang</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>张昱莹</t>
+          <t>李丹阳</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -2251,12 +2271,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
-        </is>
+        <v>1</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -2275,7 +2290,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2300,17 +2315,17 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>仵夏炎战队</t>
+          <t>李少辉战队</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>chenxiangru</t>
+          <t>yangxiju</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>陈湘茹</t>
+          <t>杨喜菊</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -2338,7 +2353,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -2363,17 +2378,17 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>李丹阳战队</t>
+          <t>王梦迪战队</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>lidanyang</t>
+          <t>zhangyuying01</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>李丹阳</t>
+          <t>张昱莹</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -2382,7 +2397,12 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
+        </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -2401,7 +2421,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -2426,17 +2446,17 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>王梦迪战队</t>
+          <t>仵夏炎战队</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>wangmengdi01</t>
+          <t>peifang</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>王梦迪</t>
+          <t>裴芳</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -2469,7 +2489,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2499,12 +2519,12 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>fansilu</t>
+          <t>zhouyingying01</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>樊思路</t>
+          <t>周莹莹</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -2532,7 +2552,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -2600,7 +2620,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -2625,17 +2645,17 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>仵夏炎战队</t>
+          <t>李少辉战队</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>zhouyingying01</t>
+          <t>lishaohui</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>周莹莹</t>
+          <t>李少辉</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -2644,7 +2664,12 @@
         </is>
       </c>
       <c r="K8" t="n">
-        <v>1</v>
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>6,7,8,9,10,11</t>
+        </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -2663,7 +2688,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2688,17 +2713,17 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>李少辉战队</t>
+          <t>仵夏炎战队</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>lijingzhe</t>
+          <t>fansilu</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>李京哲</t>
+          <t>樊思路</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -2726,7 +2751,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -2751,17 +2776,17 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>李丹阳战队</t>
+          <t>仵夏炎战队</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>zhangyali</t>
+          <t>wangchangfei</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>张亚丽</t>
+          <t>王常菲</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -2794,7 +2819,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -2824,12 +2849,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>lvzhiheng</t>
+          <t>zhangbiyu</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>吕志恒</t>
+          <t>张碧玉</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -2838,7 +2863,12 @@
         </is>
       </c>
       <c r="K11" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
+        </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
@@ -2857,7 +2887,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2882,17 +2912,17 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>李少辉战队</t>
+          <t>吕志恒战队</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>lishaohui</t>
+          <t>liudonghui</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>李少辉</t>
+          <t>刘栋辉</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -2901,7 +2931,12 @@
         </is>
       </c>
       <c r="K12" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
+        </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
@@ -2920,7 +2955,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2945,17 +2980,17 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>仵夏炎战队</t>
+          <t>王梦迪战队</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>wuxiayan</t>
+          <t>wangmengdi01</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>仵夏炎</t>
+          <t>王梦迪</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -2988,7 +3023,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -3013,17 +3048,17 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>仵夏炎战队</t>
+          <t>李丹阳战队</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>wangxinran</t>
+          <t>zhangyali</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>王欣冉</t>
+          <t>张亚丽</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -3056,7 +3091,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -3081,17 +3116,17 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>仵夏炎战队</t>
+          <t>李少辉战队</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>qinshunan</t>
+          <t>lijingzhe</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>秦淑楠</t>
+          <t>李京哲</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -3100,12 +3135,7 @@
         </is>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
-        </is>
+        <v>1</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
@@ -3124,7 +3154,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -3149,17 +3179,17 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>吕志恒战队</t>
+          <t>仵夏炎战队</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>liudonghui</t>
+          <t>wuxiayan</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>刘栋辉</t>
+          <t>仵夏炎</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -3192,7 +3222,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -3217,17 +3247,17 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>李少辉战队</t>
+          <t>仵夏炎战队</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>yangxiju</t>
+          <t>qinshunan</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>杨喜菊</t>
+          <t>秦淑楠</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -3236,7 +3266,12 @@
         </is>
       </c>
       <c r="K17" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
+        </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
@@ -3255,7 +3290,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -3285,12 +3320,12 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>peifang</t>
+          <t>wangxinran</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>裴芳</t>
+          <t>王欣冉</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -3323,7 +3358,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -3348,17 +3383,17 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>仵夏炎战队</t>
+          <t>吕志恒战队</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>wangchangfei</t>
+          <t>lvzhiheng</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>王常菲</t>
+          <t>吕志恒</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -3367,12 +3402,7 @@
         </is>
       </c>
       <c r="K19" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
-        </is>
+        <v>1</v>
       </c>
       <c r="M19" t="inlineStr">
         <is>
@@ -3391,7 +3421,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -3416,17 +3446,17 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>魏新卓战队</t>
+          <t>仵夏炎战队</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>zhangbiyu</t>
+          <t>chenxiangru</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>张碧玉</t>
+          <t>陈湘茹</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -3435,12 +3465,7 @@
         </is>
       </c>
       <c r="K20" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
-        </is>
+        <v>1</v>
       </c>
       <c r="M20" t="inlineStr">
         <is>
@@ -3464,7 +3489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3479,7 +3504,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>风灵在线未达标名单（小短）-7月23日（低价课）</t>
+          <t>风灵在线未达标名单（小短）-7月24日（低价课）</t>
         </is>
       </c>
     </row>
@@ -3719,22 +3744,22 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>吕志恒战队</t>
+          <t>仵夏炎战队</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>刘栋辉</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" s="6" t="n">
-        <v>0</v>
+          <t>陈湘茹</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>0.7777777777777778</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -3750,16 +3775,16 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>李丹阳战队</t>
+          <t>吕志恒战队</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>张亚丽</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="n">
-        <v>1</v>
+          <t>刘栋辉</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>1</v>
@@ -3781,12 +3806,12 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>王梦迪战队</t>
+          <t>吕志恒战队</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>张昱莹</t>
+          <t>张碧玉</t>
         </is>
       </c>
       <c r="E11" s="6" t="n">
@@ -3812,12 +3837,12 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>王梦迪战队</t>
+          <t>李丹阳战队</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>王梦迪</t>
+          <t>张亚丽</t>
         </is>
       </c>
       <c r="E12" s="5" t="n">
@@ -3843,21 +3868,83 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>魏新卓战队</t>
+          <t>李少辉战队</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>张碧玉</t>
+          <t>李少辉</t>
         </is>
       </c>
       <c r="E13" s="6" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>0.9444444444444444</v>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>王梦迪战队</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>张昱莹</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="F13" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G13" s="6" t="n">
+      <c r="F14" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>王梦迪战队</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>王梦迪</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="6" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Backfill weekly history 2026-08-31 through 2026-09-06.
Update dashboard and daily Excel outputs from Sep 8 source exports.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/每日输出/小短/郑州-小短-每日风灵不在线.xlsx
+++ b/每日输出/小短/郑州-小短-每日风灵不在线.xlsx
@@ -103,10 +103,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X13"/>
+  <dimension ref="A1:X19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -601,7 +601,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>20260828</v>
+        <v>20260904</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -625,7 +625,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1688855324790528</t>
+          <t>1688856448789579</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -635,22 +635,22 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>仵夏炎战队</t>
+          <t>仵夏炎</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>汪春玖</t>
+          <t>仵夏炎</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>wangchunjiu</t>
+          <t>wuxiayan</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -662,12 +662,7 @@
         <v>1</v>
       </c>
       <c r="O2" t="n">
-        <v>0.7777777777777778</v>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>9,10,11,12</t>
-        </is>
+        <v>1</v>
       </c>
       <c r="Q2" t="n">
         <v>1</v>
@@ -679,12 +674,12 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>汪春玖</t>
+          <t>仵夏炎</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>wangchunjiu</t>
+          <t>wuxiayan</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
@@ -705,7 +700,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>20260828</v>
+        <v>20260904</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -729,7 +724,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1688854644796118</t>
+          <t>1688857774777312</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -739,22 +734,22 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>王梦迪战队</t>
+          <t>秦淑楠</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>张昱莹</t>
+          <t>秦淑楠</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>zhangyuying01</t>
+          <t>qinshunan</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -763,13 +758,28 @@
         </is>
       </c>
       <c r="M3" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
+        </is>
       </c>
       <c r="O3" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
+        </is>
       </c>
       <c r="Q3" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
+        </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -778,12 +788,12 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>张昱莹</t>
+          <t>秦淑楠</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>zhangyuying01</t>
+          <t>qinshunan</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -804,7 +814,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>20260828</v>
+        <v>20260904</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -828,7 +838,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1688858172724149</t>
+          <t>1688856227810743</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -838,22 +848,22 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>吕志恒战队</t>
+          <t>仵夏炎</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>吕志恒</t>
+          <t>陈湘茹</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>lvzhiheng</t>
+          <t>chenxiangru</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -865,12 +875,7 @@
         <v>1</v>
       </c>
       <c r="O4" t="n">
-        <v>0.8888888888888888</v>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>11,12</t>
-        </is>
+        <v>1</v>
       </c>
       <c r="Q4" t="n">
         <v>1</v>
@@ -882,12 +887,12 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>吕志恒</t>
+          <t>陈湘茹</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>lvzhiheng</t>
+          <t>chenxiangru</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
@@ -908,7 +913,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>20260828</v>
+        <v>20260904</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -932,7 +937,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1688857053845933</t>
+          <t>1688855425700511</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -942,22 +947,22 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>仵夏炎战队</t>
+          <t>秦淑楠</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>裴芳</t>
+          <t>李丹阳</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>peifang</t>
+          <t>lidanyang</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -981,12 +986,12 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>裴芳</t>
+          <t>李丹阳</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>peifang</t>
+          <t>lidanyang</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
@@ -1007,7 +1012,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>20260828</v>
+        <v>20260904</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1031,7 +1036,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1688854619909919</t>
+          <t>1688855324790528</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -1041,22 +1046,22 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>吕志恒战队</t>
+          <t>仵夏炎</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>刘栋辉</t>
+          <t>汪春玖</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>liudonghui</t>
+          <t>wangchunjiu</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -1068,11 +1073,11 @@
         <v>1</v>
       </c>
       <c r="O6" t="n">
-        <v>0</v>
+        <v>0.9444444444444444</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
+          <t>11</t>
         </is>
       </c>
       <c r="Q6" t="n">
@@ -1085,12 +1090,12 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>刘栋辉</t>
+          <t>汪春玖</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>liudonghui</t>
+          <t>wangchunjiu</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
@@ -1111,7 +1116,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>20260828</v>
+        <v>20260904</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -1135,7 +1140,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>1688855425700511</t>
+          <t>1688858040865393</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1145,22 +1150,22 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>李丹阳战队</t>
+          <t>仵夏炎</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>李丹阳</t>
+          <t>王欣冉</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>lidanyang</t>
+          <t>wangxinran</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -1184,12 +1189,12 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>李丹阳</t>
+          <t>王欣冉</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>lidanyang</t>
+          <t>wangxinran</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
@@ -1210,7 +1215,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>20260828</v>
+        <v>20260904</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -1244,12 +1249,12 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>仵夏炎战队</t>
+          <t>仵夏炎</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -1309,7 +1314,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>20260828</v>
+        <v>20260904</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1333,7 +1338,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>1688854397763628</t>
+          <t>1688854876688129</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1343,22 +1348,22 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>李少辉战队</t>
+          <t>秦淑楠</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>李京哲</t>
+          <t>王梦迪</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>lijingzhe</t>
+          <t>wangmengdi01</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1382,12 +1387,12 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>李京哲</t>
+          <t>王梦迪</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>lijingzhe</t>
+          <t>wangmengdi01</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
@@ -1408,7 +1413,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>20260828</v>
+        <v>20260904</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1432,7 +1437,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>1688856227810743</t>
+          <t>1688854426767496</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1442,22 +1447,22 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>仵夏炎战队</t>
+          <t>秦淑楠</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>陈湘茹</t>
+          <t>杨喜菊</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>chenxiangru</t>
+          <t>yangxiju</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1481,12 +1486,12 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>陈湘茹</t>
+          <t>杨喜菊</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>chenxiangru</t>
+          <t>yangxiju</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
@@ -1507,7 +1512,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>20260828</v>
+        <v>20260904</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1531,7 +1536,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>1688856448789579</t>
+          <t>1688855001729445</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1541,22 +1546,22 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>仵夏炎战队</t>
+          <t>秦淑楠</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>仵夏炎</t>
+          <t>李少辉</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>wuxiayan</t>
+          <t>lishaohui</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1580,12 +1585,12 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>仵夏炎</t>
+          <t>李少辉</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>wuxiayan</t>
+          <t>lishaohui</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
@@ -1606,7 +1611,7 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>20260828</v>
+        <v>20260904</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1630,7 +1635,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1688858040865393</t>
+          <t>1688854644796118</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1640,22 +1645,22 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>仵夏炎战队</t>
+          <t>秦淑楠</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>王欣冉</t>
+          <t>张昱莹</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>wangxinran</t>
+          <t>zhangyuying01</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1670,7 +1675,12 @@
         <v>1</v>
       </c>
       <c r="Q12" t="n">
-        <v>1</v>
+        <v>0.9444444444444444</v>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
@@ -1679,12 +1689,12 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>王欣冉</t>
+          <t>张昱莹</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>wangxinran</t>
+          <t>zhangyuying01</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
@@ -1705,7 +1715,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>20260828</v>
+        <v>20260904</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1729,7 +1739,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1688854876688129</t>
+          <t>1688857053845933</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1739,22 +1749,22 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>王梦迪战队</t>
+          <t>仵夏炎</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>王梦迪</t>
+          <t>裴芳</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>wangmengdi01</t>
+          <t>peifang</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1778,12 +1788,12 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>王梦迪</t>
+          <t>裴芳</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>wangmengdi01</t>
+          <t>peifang</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
@@ -1797,6 +1807,630 @@
         </is>
       </c>
       <c r="X13" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>20260904</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>短期班</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>初中</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>1688855018925954</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>秦淑楠</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>温玉璇</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>wenyuxuan</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>低价课</t>
+        </is>
+      </c>
+      <c r="M14" t="n">
+        <v>1</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
+        </is>
+      </c>
+      <c r="Q14" t="n">
+        <v>1</v>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>温玉璇</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>wenyuxuan</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>20260904</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>短期班</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>1688854397763628</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>秦淑楠</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>李京哲</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>lijingzhe</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>低价课</t>
+        </is>
+      </c>
+      <c r="M15" t="n">
+        <v>1</v>
+      </c>
+      <c r="O15" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>1</v>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>李京哲</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>lijingzhe</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>20260904</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>短期班</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>1688856042840562</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>秦淑楠</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>王聪阳</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>wangcongyang</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>低价课</t>
+        </is>
+      </c>
+      <c r="M16" t="n">
+        <v>1</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
+        </is>
+      </c>
+      <c r="Q16" t="n">
+        <v>1</v>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>王聪阳</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>wangcongyang</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>20260904</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>短期班</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>1688858172724149</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>仵夏炎</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>吕志恒</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>lvzhiheng</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>低价课</t>
+        </is>
+      </c>
+      <c r="M17" t="n">
+        <v>1</v>
+      </c>
+      <c r="O17" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>1</v>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>吕志恒</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>lvzhiheng</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>20260904</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>短期班</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>初中</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>1688855861872405</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>仵夏炎</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>张碧玉</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>zhangbiyu</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>低价课</t>
+        </is>
+      </c>
+      <c r="M18" t="n">
+        <v>1</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
+        </is>
+      </c>
+      <c r="Q18" t="n">
+        <v>1</v>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>张碧玉</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>zhangbiyu</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>20260904</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>短期班</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>1688854619909919</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>仵夏炎</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>刘栋辉</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>liudonghui</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>低价课</t>
+        </is>
+      </c>
+      <c r="M19" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>6,7,8,9,10,11</t>
+        </is>
+      </c>
+      <c r="O19" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
+        </is>
+      </c>
+      <c r="Q19" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>6,7,8,9,10,11</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>刘栋辉</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>liudonghui</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
         <is>
           <t>小短</t>
         </is>
@@ -1813,1139 +2447,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R13"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>服务期</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>日期</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>学段</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>分部</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>阶段</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>运营中心</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>战队</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>学习规划师</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>学习规划师姓名</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>带班产品</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>风灵微信在线率</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>不在线时段list</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>年级</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>学部</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>辅导老师</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>辅导姓名</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>sys_source</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>分组</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>20260828</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>爱学</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>短期班</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>全年级</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>郑州</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>王梦迪战队</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>wangmengdi01</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>王梦迪</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>低价课</t>
-        </is>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>全年级</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>小学</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>wangmengdi01</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>王梦迪</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>爱学</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>小短</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>20260828</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>爱学</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>短期班</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>全年级</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>郑州</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>仵夏炎战队</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>chenxiangru</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>陈湘茹</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>低价课</t>
-        </is>
-      </c>
-      <c r="K3" t="n">
-        <v>1</v>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>全年级</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>小学</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>chenxiangru</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>陈湘茹</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>爱学</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>小短</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>20260828</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>爱学</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>短期班</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>全年级</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>郑州</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>吕志恒战队</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>lvzhiheng</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>吕志恒</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>低价课</t>
-        </is>
-      </c>
-      <c r="K4" t="n">
-        <v>0.8888888888888888</v>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>11,12</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>全年级</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>小学</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>lvzhiheng</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>吕志恒</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>爱学</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>小短</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>20260828</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>爱学</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>短期班</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>全年级</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>郑州</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>仵夏炎战队</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>wangchunjiu</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>汪春玖</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>低价课</t>
-        </is>
-      </c>
-      <c r="K5" t="n">
-        <v>0.7777777777777778</v>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>9,10,11,12</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>全年级</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>小学</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>wangchunjiu</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>汪春玖</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>爱学</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>小短</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>20260828</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>爱学</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>短期班</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>全年级</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>郑州</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>王梦迪战队</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>zhangyuying01</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>张昱莹</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>低价课</t>
-        </is>
-      </c>
-      <c r="K6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>全年级</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>小学</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>zhangyuying01</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>张昱莹</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>爱学</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>小短</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>20260828</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>爱学</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>短期班</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>全年级</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>郑州</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>仵夏炎战队</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>jingyabo</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>荆雅博</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>低价课</t>
-        </is>
-      </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>全年级</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>小学</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>jingyabo</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>荆雅博</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>爱学</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>小短</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>20260828</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>爱学</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>短期班</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>全年级</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>郑州</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>仵夏炎战队</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>wangxinran</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>王欣冉</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>低价课</t>
-        </is>
-      </c>
-      <c r="K8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>全年级</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>小学</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>wangxinran</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>王欣冉</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>爱学</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>小短</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>20260828</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>爱学</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>短期班</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>全年级</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>郑州</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>仵夏炎战队</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>peifang</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>裴芳</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>低价课</t>
-        </is>
-      </c>
-      <c r="K9" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>全年级</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>小学</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>peifang</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>裴芳</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>爱学</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>小短</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>20260828</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>爱学</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>短期班</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>全年级</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>郑州</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>李丹阳战队</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>lidanyang</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>李丹阳</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>低价课</t>
-        </is>
-      </c>
-      <c r="K10" t="n">
-        <v>1</v>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>全年级</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>小学</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>lidanyang</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>李丹阳</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>爱学</t>
-        </is>
-      </c>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>小短</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>20260828</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>爱学</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>短期班</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>全年级</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>郑州</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>吕志恒战队</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>liudonghui</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>刘栋辉</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>低价课</t>
-        </is>
-      </c>
-      <c r="K11" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>全年级</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>小学</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>liudonghui</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>刘栋辉</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>爱学</t>
-        </is>
-      </c>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>小短</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>20260828</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>爱学</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>短期班</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>全年级</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>郑州</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>仵夏炎战队</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>wuxiayan</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>仵夏炎</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>低价课</t>
-        </is>
-      </c>
-      <c r="K12" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>全年级</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>小学</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>wuxiayan</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>仵夏炎</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>爱学</t>
-        </is>
-      </c>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>小短</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>20260828</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>爱学</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>短期班</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>全年级</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>郑州</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>李少辉战队</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>lijingzhe</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>李京哲</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>低价课</t>
-        </is>
-      </c>
-      <c r="K13" t="n">
-        <v>1</v>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>全年级</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>小学</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>lijingzhe</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>李京哲</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>爱学</t>
-        </is>
-      </c>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>小短</t>
+          <t>无数据</t>
         </is>
       </c>
     </row>
@@ -2960,7 +2468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2975,7 +2483,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>风灵在线未达标名单（小短）-8月27日（低价课）</t>
+          <t>风灵在线未达标名单（小短）-9月6日（低价课）</t>
         </is>
       </c>
     </row>
@@ -3029,22 +2537,22 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>仵夏炎战队</t>
+          <t>仵夏炎</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>仵夏炎</t>
+          <t>刘栋辉</t>
         </is>
       </c>
       <c r="E3" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G3" s="6" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="G3" s="3" t="e">
+        <v>#N/A</v>
       </c>
     </row>
     <row r="4">
@@ -3060,22 +2568,22 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>仵夏炎战队</t>
+          <t>仵夏炎</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>汪春玖</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="n">
-        <v>0.7777777777777778</v>
-      </c>
-      <c r="F4" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G4" s="6" t="n">
-        <v>0.7777777777777778</v>
+          <t>张碧玉</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" s="3" t="e">
+        <v>#N/A</v>
       </c>
     </row>
     <row r="5">
@@ -3091,22 +2599,22 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>仵夏炎战队</t>
+          <t>仵夏炎</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>王欣冉</t>
+          <t>汪春玖</t>
         </is>
       </c>
       <c r="E5" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F5" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" s="6" t="n">
-        <v>0</v>
+        <v>0.9444444444444444</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="3" t="e">
+        <v>#N/A</v>
       </c>
     </row>
     <row r="6">
@@ -3122,22 +2630,22 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>仵夏炎战队</t>
+          <t>秦淑楠</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>荆雅博</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="n">
+          <t>张昱莹</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G6" s="6" t="n">
-        <v>0</v>
+        <v>0.9444444444444444</v>
+      </c>
+      <c r="G6" s="3" t="e">
+        <v>#N/A</v>
       </c>
     </row>
     <row r="7">
@@ -3153,22 +2661,22 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>仵夏炎战队</t>
+          <t>秦淑楠</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>裴芳</t>
+          <t>温玉璇</t>
         </is>
       </c>
       <c r="E7" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F7" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" s="6" t="n">
         <v>0</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="3" t="e">
+        <v>#N/A</v>
       </c>
     </row>
     <row r="8">
@@ -3184,22 +2692,22 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>吕志恒战队</t>
+          <t>秦淑楠</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>刘栋辉</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="n">
+          <t>王聪阳</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F8" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" s="6" t="n">
-        <v>0</v>
+      <c r="F8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="3" t="e">
+        <v>#N/A</v>
       </c>
     </row>
     <row r="9">
@@ -3215,84 +2723,22 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>吕志恒战队</t>
+          <t>秦淑楠</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>吕志恒</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="n">
-        <v>0.8888888888888888</v>
+          <t>秦淑楠</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" s="6" t="n">
-        <v>0.8888888888888888</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>小学</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>全年级</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>王梦迪战队</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>张昱莹</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F10" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G10" s="6" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>小学</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>全年级</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>王梦迪战队</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>王梦迪</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F11" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G11" s="6" t="n">
-        <v>0</v>
+      <c r="G9" s="3" t="e">
+        <v>#N/A</v>
       </c>
     </row>
   </sheetData>

</xml_diff>